<commit_message>
P3 step 2: vendor products, price lists, vendor comparison (DL-157..159)
- Vendor code, unit, cost and currency per product; one preferred vendor; previous cost kept
- Price list import (CSV/Excel in the browser) matched by vendor code then barcode
- Compare vendors in CAD per base unit; better prices list; Buying screen
- Permissions purchasing.view / purchasing.manage; tests step33 (18); sample vendor prices

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -805,9 +805,219 @@
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Vendor prices</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Buying → Vendor prices → Coastal Beverages</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>The sample products with unit, code, cost; ★ on preferred ones</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Vendor prices</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Add a product: chips, comes as the largest unit, cost, preferred</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Saved; any other vendor's ★ for chips goes</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Vendor prices</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Change its cost</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Shows 'was …' in red (up) or green (down)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Price list</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Import price list: an Excel file with Code, Barcode, Description, Price columns (one unknown barcode, one empty price)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Columns guessed; result: new / changed / same, up and down lists, two rows not matched with the reason</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Compare</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Phone (staff)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Compare vendors → chips</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Maple (USD) and Coastal with the cost per base unit in CAD; cheapest marked</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Compare</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Better prices</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Products whose ★ vendor is not the cheapest, with −%</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
-  <conditionalFormatting sqref="F2:F7">
+  <autoFilter ref="A1:I13"/>
+  <conditionalFormatting sqref="F2:F13">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -822,7 +1032,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -836,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -907,29 +1117,110 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Vendor prices</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>COUNTIF(Tests!B:B,A3)</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Price list</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(Tests!B:B,A4)</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Compare</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF(Tests!B:B,A5)</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B3" s="5">
-        <f>SUM(B2:B2)</f>
-        <v/>
-      </c>
-      <c r="C3" s="5">
-        <f>SUM(C2:C2)</f>
-        <v/>
-      </c>
-      <c r="D3" s="5">
-        <f>SUM(D2:D2)</f>
-        <v/>
-      </c>
-      <c r="E3" s="5">
-        <f>SUM(E2:E2)</f>
-        <v/>
-      </c>
-      <c r="F3" s="5">
-        <f>SUM(F2:F2)</f>
+      <c r="B6" s="5">
+        <f>SUM(B2:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>SUM(C2:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>SUM(D2:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>SUM(E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>SUM(F2:F5)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 3: purchase orders, receiving against them, min/max reorder (DL-160..162)
- Draft / send (PDF) / receive partly or fully / close / cancel; incoming stock
- Receiving through the P1 receive action at the PO's exchange rate; differences flagged with a task
- Reorder point + order-up-to max make draft POs per vendor
- Tests step34 (24)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1015,9 +1015,254 @@
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Q20</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Buying → New order: Coastal, two products from 'Add what this vendor sells', change a quantity</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Draft PO-… with the vendor's costs and the total</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Q21</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Send</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Status Sent; a PDF downloads with the store, vendor, lines and total; Stock shows the quantity as incoming</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Q22</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Phone (staff)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Open the order → Receive: part of one line</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Partly received; stock goes up; incoming goes down</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Q23</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Phone (staff)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Receive the rest with a higher cost on one line and one more than ordered</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Received; differences 'different cost', 'more than ordered'; a task for the managers</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Q24</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Another order: receive part, tick 'The rest will not come'</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Closed; 'short' shown; incoming back down</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Q25</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Order from Maple Snacks (USD)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Shows USD, the rate and the CAD total</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Q26</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Reorder</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>A product: reorder when stock falls to 50, order up to 100 (above its stock)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Purchase orders lists it; Make the orders makes a draft for its vendor in whole cases up to 100</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
-  <conditionalFormatting sqref="F2:F13">
+  <autoFilter ref="A1:I20"/>
+  <conditionalFormatting sqref="F2:F20">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1032,7 +1277,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1046,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1198,29 +1443,83 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>COUNTIF(Tests!B:B,A6)</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Reorder</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>COUNTIF(Tests!B:B,A7)</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B6" s="5">
-        <f>SUM(B2:B5)</f>
-        <v/>
-      </c>
-      <c r="C6" s="5">
-        <f>SUM(C2:C5)</f>
-        <v/>
-      </c>
-      <c r="D6" s="5">
-        <f>SUM(D2:D5)</f>
-        <v/>
-      </c>
-      <c r="E6" s="5">
-        <f>SUM(E2:E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="5">
-        <f>SUM(F2:F5)</f>
+      <c r="B8" s="5">
+        <f>SUM(B2:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>SUM(C2:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>SUM(D2:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>SUM(F2:F7)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 4: bills, invoices, payments, statements, vendor returns, performance (DL-163..166)
- Payables and receivables with currency, rate, taxes, due dates, photos; aging
- Payments incl. applying credits; statements with PDF; bill from a received PO (three-way)
- Returns to vendors take stock out at cost; vendor credit; vendor performance
- Permission finance.manage (managers, accountant); tests step35 (26)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1260,9 +1260,324 @@
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Q30</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Buying → Bills and invoices → New bill: Coastal, their no. CB-1, two lines, GST, a photo</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>B-… open, due from Coastal's 30 days, total with tax; the photo opens</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Q31</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Record a payment: part by cheque with its number</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Partly paid; the rest shown; the cheque on the bill</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Q32</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Vendor credit for Coastal, then apply it to the bill</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>The credit is used; the bill's balance goes down</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Q33</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Take the credit payment off</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>The bill and the credit are open again</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Q34</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Invoices</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Owed to us → New invoice to Cafe Luna; record money received</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>INV-…; aging; Statement shows invoice, payment, balance; PDF</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Q35</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>A received PO → Make the bill from what was received</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>A bill with the received quantities; a bill for more than received says 'above what was received'</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Q36</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Vendor returns</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Returns to vendors → Send goods back: 2 damaged chips, RMA</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>VR-…; stock down by 2 at once; Record their credit makes a vendor credit</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Q37</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Vendor returns</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Vendor performance</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>On time, short and damaged % for vendors with received orders</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Q38</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Phone (staff)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Buying as Sam Staff</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>No Bills and invoices tab</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I20"/>
-  <conditionalFormatting sqref="F2:F20">
+  <autoFilter ref="A1:I29"/>
+  <conditionalFormatting sqref="F2:F29">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1277,7 +1592,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1291,7 +1606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1497,29 +1812,110 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(Tests!B:B,A8)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Invoices</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(Tests!B:B,A9)</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Vendor returns</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTIF(Tests!B:B,A10)</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B8" s="5">
-        <f>SUM(B2:B7)</f>
-        <v/>
-      </c>
-      <c r="C8" s="5">
-        <f>SUM(C2:C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="5">
-        <f>SUM(D2:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="5">
-        <f>SUM(E2:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="5">
-        <f>SUM(F2:F7)</f>
+      <c r="B11" s="5">
+        <f>SUM(B2:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>SUM(C2:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="5">
+        <f>SUM(D2:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="5">
+        <f>SUM(E2:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>SUM(F2:F10)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 5: receive from a bill photo or PDF, landed cost (DL-167..169)
- Bills read on the device (Tesseract served by the hub, pdf.js), parsed into lines and totals with checks
- Hub matching: learned, vendor code, barcode, name; open order check; review grid
- Receiving with freight/duty/brokerage spread by value (also on PO receipts); learns matches; records the bill
- Tests step36 (17)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1575,9 +1575,219 @@
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Q40</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Bill photo</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>iPhone (staff)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Add stock → read the vendor's bill → Coastal → 📷 a printed bill</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>'Reading the photo…', then the lines with products matched (their code / barcode / by name) and the totals</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Q41</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Bill photo</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>iPhone</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>A line not matched: type to search, pick the product</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Matched; Receive into stock adds the stock</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Q42</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Bill photo</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>iPhone</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Another bill from Coastal with the same item</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>That line is matched by itself ('remembered')</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Q43</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Bill photo</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>A PDF bill for an open order; freight on the bill; tick 'Also record the bill'</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Order suggested, lines 'as ordered'; freight filled in; order received; bill B-… with freight as a line</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Q44</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Landed cost</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Receive an order by hand with Freight 10.00</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Each item's cost (Stock → the product → lots) includes its share of the $10 by value</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Q45</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Bill photo</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>A bill whose lines do not add up</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>A warning saying by how much</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
+      <c r="H35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I29"/>
-  <conditionalFormatting sqref="F2:F29">
+  <autoFilter ref="A1:I35"/>
+  <conditionalFormatting sqref="F2:F35">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1592,7 +1802,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1606,7 +1816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1893,29 +2103,83 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bill photo</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(Tests!B:B,A11)</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Landed cost</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>COUNTIF(Tests!B:B,A12)</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B11" s="5">
-        <f>SUM(B2:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="5">
-        <f>SUM(C2:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="5">
-        <f>SUM(D2:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="5">
-        <f>SUM(E2:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="5">
-        <f>SUM(F2:F10)</f>
+      <c r="B13" s="5">
+        <f>SUM(B2:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>SUM(C2:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="5">
+        <f>SUM(D2:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="5">
+        <f>SUM(E2:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>SUM(F2:F12)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 6: expenses and petty cash (DL-170..172)
- Claims with receipt photos, GST/PST, categories; approve/reject; pay back (till pay-out, petty cash, cheque, e-transfer, next pay)
- Duplicate and missing-receipt flags; petty cash box with top-ups and counts
- Permission expenses.approve (managers, accountant); tests step37 (19)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1785,9 +1785,219 @@
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr"/>
     </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Q50</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>iPhone (staff)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Expenses → New claim: Home Depot, $23.50 with GST, own money, 📷 the receipt</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>EX-… waiting; shown under My claims with the photo</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Q51</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Till (cashier)</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>The same amount and place without a photo</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Flags: 'same as EX-…?' and 'no receipt photo'</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Q52</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>All claims: reject the duplicate with a reason; approve the first</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Rejected / Approved, to pay back</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
+      <c r="H38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Q53</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Pay back → Cash from the till (a till is open)</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Done; the till's Z report shows the pay-out</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Q54</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Your own claim: Approve</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Refused: someone else approves it</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Q55</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Petty cash</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Petty cash → Top up 200; a claim paid from the box (5.00); Count 194.00</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Box 200 → 195 → count 'Short 1.00', balance 194</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I35"/>
-  <conditionalFormatting sqref="F2:F35">
+  <autoFilter ref="A1:I41"/>
+  <conditionalFormatting sqref="F2:F41">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1802,7 +2012,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1816,7 +2026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2157,29 +2367,83 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>COUNTIF(Tests!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Petty cash</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>COUNTIF(Tests!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B13" s="5">
-        <f>SUM(B2:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="5">
-        <f>SUM(C2:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="5">
-        <f>SUM(D2:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="5">
-        <f>SUM(E2:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="5">
-        <f>SUM(F2:F12)</f>
+      <c r="B15" s="5">
+        <f>SUM(B2:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="5">
+        <f>SUM(C2:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="5">
+        <f>SUM(D2:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="5">
+        <f>SUM(E2:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>SUM(F2:F14)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 7: layaway, special orders, quotes, house accounts (DL-173..177)
- Client orders with reserved stock, deposits/refunds at the till (counted in the drawer and card totals)
- Ring up at the till: agreed prices, Deposit payment applied by the hub; order picked up in the sale
- Quotes expire; become layaway, special order or invoice; On account payment makes an invoice within the credit limit
- Tests step38 (21); sales, offline and returns suites still pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1995,9 +1995,254 @@
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Q60</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Layaway</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Customer orders → New layaway: Rita, phone, 2 items, deposit 20% cash</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>LA-… open, goods kept aside (Stock shows reserved); the till's expected cash includes the deposit</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr"/>
+      <c r="H42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Q61</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Layaway</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Take a payment by card; then Ring up at the till</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Sell shows the order's lines and 'the deposit … is used'; Pay starts with Deposit; finish by card; the order is Picked up</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr"/>
+      <c r="H43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Q62</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Layaway</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Another layaway → Cancel → give the deposit back in cash</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Cancelled; the drawer's expected cash goes down; reservation released</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Q63</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Special order</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>New special order (24 chocolate bars) → Ordered → Arrived</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Ready for pickup; reserved only once arrived; Ring up works then</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Q64</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>New quote for Cafe Luna at a lower agreed price; PDF; Make it an invoice</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>QT-… PDF; turned into INV-… for Luna</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Q65</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>A quote → Ring up at the till</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>The agreed price shows as an override with the quote as the reason</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Q66</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>House account</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Sell → Pay → On account → Cafe Luna</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Sale done; an invoice INV-… for Luna (Bills and invoices); over the limit is refused</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I41"/>
-  <conditionalFormatting sqref="F2:F41">
+  <autoFilter ref="A1:I48"/>
+  <conditionalFormatting sqref="F2:F48">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2012,7 +2257,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2026,7 +2271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2421,29 +2666,137 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Layaway</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(Tests!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Special order</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>COUNTIF(Tests!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>COUNTIF(Tests!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>House account</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>COUNTIF(Tests!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B15" s="5">
-        <f>SUM(B2:B14)</f>
-        <v/>
-      </c>
-      <c r="C15" s="5">
-        <f>SUM(C2:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="5">
-        <f>SUM(D2:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="5">
-        <f>SUM(E2:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="5">
-        <f>SUM(F2:F14)</f>
+      <c r="B19" s="5">
+        <f>SUM(B2:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>SUM(C2:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="5">
+        <f>SUM(D2:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="5">
+        <f>SUM(E2:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="5">
+        <f>SUM(F2:F18)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 8: bundles, variants, serial numbers (DL-178..180)
- Bundles take components out of stock (sale, offline upload, return); availability
- Variants made from a parent's axes; till asks which variant
- Serial/IMEI per unit at the sale, never sold twice; warranty lookup
- Tests step39 (18); sales, offline, returns, pricing suites pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2240,9 +2240,254 @@
       <c r="H48" s="3" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr"/>
     </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Q70</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Bundles</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Products → New: 'Movie night kit', Bundle or kit: chips ×1 + chocolate ×2, barcode, price; activate</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Saved; the components listed</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Q71</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Bundles</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Sell 2 kits</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Stock: chips −2, chocolate −4 (the kit itself has no stock); too many kits for the stock is refused</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Q72</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Bundles</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Return 1 kit to stock</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Chips +1, chocolate +2</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr"/>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Q73</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Variants</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>A product → Variety → Variants: Size S, M, L; Colour Black, White → Make the variants</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>6 variants as drafts; adding XL later makes 2 more</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr"/>
+      <c r="H52" s="3" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Q74</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Variants</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Give two variants a barcode and activate them; tap the parent on the till</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Asks which one; the chosen variant goes in the cart</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr"/>
+      <c r="H53" s="3" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Q75</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Serials</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>A product with 'Serial or IMEI' (warranty 365): sell 2 without serials</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>'Scan the serial… (0 of 2)'; Enter serials; sold</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr"/>
+      <c r="H54" s="3" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Q76</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Serials</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Sell again with a serial already sold</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Refused: 'already sold'</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr"/>
+      <c r="H55" s="3" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I48"/>
-  <conditionalFormatting sqref="F2:F48">
+  <autoFilter ref="A1:I55"/>
+  <conditionalFormatting sqref="F2:F55">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2257,7 +2502,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2271,7 +2516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2774,29 +3019,110 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bundles</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>COUNTIF(Tests!B:B,A19)</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F19">
+        <f>COUNTIFS(Tests!B:B,A19,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Variants</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>COUNTIF(Tests!B:B,A20)</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F20">
+        <f>COUNTIFS(Tests!B:B,A20,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Serials</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>COUNTIF(Tests!B:B,A21)</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>COUNTIFS(Tests!B:B,A21,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D21">
+        <f>COUNTIFS(Tests!B:B,A21,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E21">
+        <f>COUNTIFS(Tests!B:B,A21,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F21">
+        <f>COUNTIFS(Tests!B:B,A21,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B19" s="5">
-        <f>SUM(B2:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="5">
-        <f>SUM(C2:C18)</f>
-        <v/>
-      </c>
-      <c r="D19" s="5">
-        <f>SUM(D2:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="5">
-        <f>SUM(E2:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="5">
-        <f>SUM(F2:F18)</f>
+      <c r="B22" s="5">
+        <f>SUM(B2:B21)</f>
+        <v/>
+      </c>
+      <c r="C22" s="5">
+        <f>SUM(C2:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="5">
+        <f>SUM(D2:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="5">
+        <f>SUM(E2:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="5">
+        <f>SUM(F2:F21)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 9: delivery-app orders (manual), consignment (DL-181, 182)
- Delivery orders: platform prices, accepted (reserved), preparing, picked up (sale paid by the platform), cancelled
- Consignment products: owed per unit sold (sales, offline, bundles, returns), not in stock value, billed per vendor
- Tests step40 (15); sales, offline, returns, dashboard, variety suites pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2485,9 +2485,219 @@
       <c r="H55" s="3" t="inlineStr"/>
       <c r="I55" s="3" t="inlineStr"/>
     </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Q80</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Delivery orders → Platform prices: Uber Eats price for chips</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Saved</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr"/>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Q81</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>New order: Uber Eats, their number, 2 chips + 1 chocolate → Accept</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Total at the Uber Eats price for chips; Stock shows them reserved</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr"/>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Q82</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Preparing → Picked up</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>A sale on this till paid by 'Platform'; reservation released; the Z report shows Platform</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr"/>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Q83</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Another order → Cancel</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Cancelled; reservation released</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr"/>
+      <c r="I59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Q84</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Consignment</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>A product → Variety → Consignment: Fresh Fields, $6.00 owed per unit; receive 10</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard stock value does not change</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr"/>
+      <c r="H60" s="3" t="inlineStr"/>
+      <c r="I60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Q85</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Consignment</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Till + laptop</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Sell 3, return 1; Buying → Consignment</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Fields: 2 sold, $12.00; Make their bill → a vendor bill, the list is empty</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
-  <conditionalFormatting sqref="F2:F55">
+  <autoFilter ref="A1:I61"/>
+  <conditionalFormatting sqref="F2:F61">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2502,7 +2712,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2516,7 +2726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3100,29 +3310,83 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>COUNTIF(Tests!B:B,A22)</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>COUNTIFS(Tests!B:B,A22,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D22">
+        <f>COUNTIFS(Tests!B:B,A22,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E22">
+        <f>COUNTIFS(Tests!B:B,A22,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F22">
+        <f>COUNTIFS(Tests!B:B,A22,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Consignment</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>COUNTIF(Tests!B:B,A23)</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>COUNTIFS(Tests!B:B,A23,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D23">
+        <f>COUNTIFS(Tests!B:B,A23,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>COUNTIFS(Tests!B:B,A23,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F23">
+        <f>COUNTIFS(Tests!B:B,A23,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B22" s="5">
-        <f>SUM(B2:B21)</f>
-        <v/>
-      </c>
-      <c r="C22" s="5">
-        <f>SUM(C2:C21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="5">
-        <f>SUM(D2:D21)</f>
-        <v/>
-      </c>
-      <c r="E22" s="5">
-        <f>SUM(E2:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="5">
-        <f>SUM(F2:F21)</f>
+      <c r="B24" s="5">
+        <f>SUM(B2:B23)</f>
+        <v/>
+      </c>
+      <c r="C24" s="5">
+        <f>SUM(C2:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="5">
+        <f>SUM(D2:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="5">
+        <f>SUM(E2:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="5">
+        <f>SUM(F2:F23)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P3 step 10: recall trace and customer feedback (DL-183..185)
- Trace lots: received, sales, members; recall writes off what is left and blocks the lots (FEFO skips them)
- Feedback from a kiosk tablet or the receipt link (coded, once per visit); report with average
- Tests step41 (17); stock, sales, markdown, printing suites pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P3.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P3.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2695,9 +2695,219 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr"/>
     </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Q90</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Receive chocolate with lot code LOT-X; sell 2 to a member; Recalls → chocolate, LOT-X → Trace</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>The lot: received, 2 sold on S-…, to the member (first name, last 4 digits)</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr"/>
+      <c r="H62" s="3" t="inlineStr"/>
+      <c r="I62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Q91</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Recall these lots with a reason</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>RC-…; what was left written off (Stock: loss 'Recall'); later sales never take that lot</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr"/>
+      <c r="H63" s="3" t="inlineStr"/>
+      <c r="I63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Q92</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Pair a tablet as a kiosk</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Shows the store's question and stars, no sign-in; Send → Thank you, then ready again</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr"/>
+      <c r="H64" s="3" t="inlineStr"/>
+      <c r="I64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Q93</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Reports → Feedback: switch on the receipt link (hub address)</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>New receipts end with 'Tell us how we did:' and a link</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Q94</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Phone on the store Wi-Fi</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Open the receipt's link; send 2 stars</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Thank you; opening it again: 'we already have your feedback'</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Q95</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Reports → Feedback</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Average, counts by stars, comments; Read clears the new mark</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr"/>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I61"/>
-  <conditionalFormatting sqref="F2:F61">
+  <autoFilter ref="A1:I67"/>
+  <conditionalFormatting sqref="F2:F67">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2712,7 +2922,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2726,7 +2936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3364,29 +3574,83 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>COUNTIF(Tests!B:B,A24)</f>
+        <v/>
+      </c>
+      <c r="C24">
+        <f>COUNTIFS(Tests!B:B,A24,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D24">
+        <f>COUNTIFS(Tests!B:B,A24,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E24">
+        <f>COUNTIFS(Tests!B:B,A24,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F24">
+        <f>COUNTIFS(Tests!B:B,A24,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>COUNTIF(Tests!B:B,A25)</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>COUNTIFS(Tests!B:B,A25,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D25">
+        <f>COUNTIFS(Tests!B:B,A25,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>COUNTIFS(Tests!B:B,A25,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>COUNTIFS(Tests!B:B,A25,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B24" s="5">
-        <f>SUM(B2:B23)</f>
-        <v/>
-      </c>
-      <c r="C24" s="5">
-        <f>SUM(C2:C23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="5">
-        <f>SUM(D2:D23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="5">
-        <f>SUM(E2:E23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="5">
-        <f>SUM(F2:F23)</f>
+      <c r="B26" s="5">
+        <f>SUM(B2:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>SUM(C2:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="5">
+        <f>SUM(D2:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="5">
+        <f>SUM(E2:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="5">
+        <f>SUM(F2:F25)</f>
         <v/>
       </c>
     </row>

</xml_diff>